<commit_message>
Crawler filled with the data
</commit_message>
<xml_diff>
--- a/services/flow-crawler/crawl-data.xlsx
+++ b/services/flow-crawler/crawl-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajhasekarungd/workspace/poc/ui-automation-solution/services/flow-crawler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FD9FB0-ADA2-2742-A97B-990D96607F25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC2FFE0-F280-9640-9064-53E1460BE180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="Credentials" sheetId="1" r:id="rId1"/>
     <sheet name="FormFills" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>page_pattern</t>
   </si>
@@ -42,6 +55,18 @@
   </si>
   <si>
     <t>Network</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>ThisIsNotAPassword</t>
+  </si>
+  <si>
+    <t>John Doe</t>
   </si>
 </sst>
 </file>
@@ -438,7 +463,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -464,6 +489,28 @@
       </c>
       <c r="C2" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed page crawler for tailwind css
</commit_message>
<xml_diff>
--- a/services/flow-crawler/crawl-data.xlsx
+++ b/services/flow-crawler/crawl-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajhasekarungd/workspace/poc/ui-automation-solution/services/flow-crawler/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC2FFE0-F280-9640-9064-53E1460BE180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1CC895-7E52-CD4C-9DA0-605D71C3E4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>page_pattern</t>
   </si>
@@ -67,6 +67,15 @@
   </si>
   <si>
     <t>John Doe</t>
+  </si>
+  <si>
+    <t>Keyword</t>
+  </si>
+  <si>
+    <t>Physician Fee Schedule</t>
+  </si>
+  <si>
+    <t>HCPCS Code</t>
   </si>
 </sst>
 </file>
@@ -463,7 +472,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -511,6 +520,28 @@
       </c>
       <c r="C4" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
+        <v>99213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>